<commit_message>
docs: add digital growth plan and 36-month financial charts
</commit_message>
<xml_diff>
--- a/docs/ChemBalance_Seed_Financial_Model.xlsx
+++ b/docs/ChemBalance_Seed_Financial_Model.xlsx
@@ -2169,7 +2169,7 @@
         <v/>
       </c>
       <c r="F9" s="26">
-        <f>'P&amp;L &amp; Cash'!F25+('Revenue Build'!F37*D9-'Revenue Build'!F37)*0.91</f>
+        <f>'P&amp;L &amp; Cash'!F25+(SUM('Revenue Build'!D37:F37)*D9-SUM('Revenue Build'!D37:F37))*0.91</f>
         <v/>
       </c>
       <c r="G9" t="inlineStr">
@@ -2192,7 +2192,7 @@
         <v/>
       </c>
       <c r="F10" s="29">
-        <f>'P&amp;L &amp; Cash'!F25+('Revenue Build'!F37*D10-'Revenue Build'!F37)*0.91</f>
+        <f>'P&amp;L &amp; Cash'!F25+(SUM('Revenue Build'!D37:F37)*D10-SUM('Revenue Build'!D37:F37))*0.91</f>
         <v/>
       </c>
       <c r="G10" s="27" t="inlineStr">
@@ -2215,7 +2215,7 @@
         <v/>
       </c>
       <c r="F11" s="26">
-        <f>'P&amp;L &amp; Cash'!F25+('Revenue Build'!F37*D11-'Revenue Build'!F37)*0.91</f>
+        <f>'P&amp;L &amp; Cash'!F25+(SUM('Revenue Build'!D37:F37)*D11-SUM('Revenue Build'!D37:F37))*0.91</f>
         <v/>
       </c>
       <c r="G11" t="inlineStr">
@@ -2236,7 +2236,7 @@
     <row r="15">
       <c r="C15" s="30" t="inlineStr">
         <is>
-          <t>The downside / base / upside cases vary only customer acquisition. Product costs, headcount, and pricing remain at base assumptions so decision-makers can see commercial sensitivity clearly.</t>
+          <t>The downside / base / upside cases vary customer acquisition across all three forecast years. Product costs, headcount, and pricing remain at base assumptions so decision-makers can see commercial sensitivity clearly.</t>
         </is>
       </c>
     </row>

</xml_diff>